<commit_message>
游戏数据：新增 1NF3S0N 与 Fly of Beelzebub
</commit_message>
<xml_diff>
--- a/qwwshs/plugins/bm/constexcel.xlsx
+++ b/qwwshs/plugins/bm/constexcel.xlsx
@@ -14622,6 +14622,109 @@
         <ns0:v>13.5</ns0:v>
       </ns0:c>
     </ns0:row>
+    <ns0:row r="248" spans="1:16">
+      <ns0:c r="A248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1NF3S+@+!0N</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DM DOKURO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>青岚柟</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>xian</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G248" s="8">
+        <ns0:v>7.0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>xian</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I248" s="8">
+        <ns0:v>10.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="J248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Swimmingtalker</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K248" s="8">
+        <ns0:v>12.0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L248" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Xi!An</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M248" s="8">
+        <ns0:v>13.0</ns0:v>
+      </ns0:c>
+      <ns0:c r="R248" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t>1NF3S0N</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="249" spans="1:16">
+      <ns0:c r="A249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fly of Beelzebub</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DM DOKURO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Frank_DL / 擦屁股的猫</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Remaine_WH被杀死了 凶手是瘟疫导弹</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G249" s="8">
+        <ns0:v>4.0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Remaine_WH奴役了蜜蜂。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I249" s="8">
+        <ns0:v>8.8</ns0:v>
+      </ns0:c>
+      <ns0:c r="J249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ICEbluebee_</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K249" s="8">
+        <ns0:v>12.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="L249" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fly of Beelzebub</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M249" s="8">
+        <ns0:v>13.2</ns0:v>
+      </ns0:c>
+    </ns0:row>
   </ns0:sheetData>
   <ns0:autoFilter ref="A1:R244">
     <ns0:sortState ref="A2:R244">

</xml_diff>